<commit_message>
Controller RC1.3: exact Samtec FTSH-105-01-L-DV-K footprint (drawing rev H), verified 1.5SMBJ12CA data, rerouted; checks clean
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/rc1_3/OSBAMS_Rev2_RC13/OSBAMS_Rev2_RC13_BOM.xlsx
+++ b/Hardware/Rev2_Controller/rc1_3/OSBAMS_Rev2_RC13/OSBAMS_Rev2_RC13_BOM.xlsx
@@ -2782,12 +2782,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>PinHeader_2x05_P1.27mm_Vertical_SMD</t>
+          <t>FTSH-105-01-L-DV-K</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Connector_PinHeader_1.27mm:PinHeader_2x05_P1.27mm_Vertical_SMD</t>
+          <t>OSBAMS_Rev2:FTSH-105-01-L-DV-K</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Bidirectional TVS 12 V standoff 1500 W (INA228 IN+/IN- differential clamp; datasheet NOT supplied, values UNVERIFIED)</t>
+          <t>Bidirectional TVS 12 V standoff 1500 W (INA228 IN+/IN- differential clamp). Bourns datasheet: VBR 13.3-14.7 V, IR 1 uA @ 12 V, VC 19.9 V @ 75.4 A (10/1000 us), 25.9 V @ 377 A (8/20 us)</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -4106,9 +4106,9 @@
           <t>Diode_SMD:D_SMB</t>
         </is>
       </c>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">

</xml_diff>